<commit_message>
Multiple updates mainly to barplot functions; pushing to v0.1.5
</commit_message>
<xml_diff>
--- a/docs/example_output/table1.xlsx
+++ b/docs/example_output/table1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -390,6 +390,33 @@
   </si>
   <si>
     <t xml:space="preserve">Solid tissue normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colon adenocarcinoma (N=522)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rectum adenocarcinoma (N=176)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age, mean±sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gender, n (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race, n (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethnicity, n (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clinical stage, n (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior treatment, n (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tissue sample type, n (%)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Multiple edits/fixes; pushing to v0.1.9
</commit_message>
<xml_diff>
--- a/docs/example_output/table1.xlsx
+++ b/docs/example_output/table1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -417,6 +417,18 @@
   </si>
   <si>
     <t xml:space="preserve">Tissue sample type, n (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">American Indian Or Alaska Native</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Or African American</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hispanic Or Latino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not Hispanic Or Latino</t>
   </si>
 </sst>
 </file>

</xml_diff>